<commit_message>
Update results with data through June 2026
</commit_message>
<xml_diff>
--- a/date_simp_concat.xlsx
+++ b/date_simp_concat.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Desktop\simpozion\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Desktop\Doctorat\simpozion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC8FC8B7-A4D4-493F-9E72-662ABEB64112}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{432710BF-29F3-45A3-BD91-BBB3BCCBB788}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -51,7 +51,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
+    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
   </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
@@ -108,7 +108,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="165" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
@@ -413,7 +413,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H3528"/>
+  <dimension ref="A1:H3613"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="18.109375" bestFit="1" customWidth="1"/>
@@ -92147,6 +92147,2216 @@
         <v>81.2</v>
       </c>
     </row>
+    <row r="3529" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3529" s="2">
+        <v>46056</v>
+      </c>
+      <c r="B3529">
+        <v>226.48</v>
+      </c>
+      <c r="C3529">
+        <v>617.92999999999995</v>
+      </c>
+      <c r="D3529">
+        <v>19.350000000000001</v>
+      </c>
+      <c r="E3529">
+        <v>2.8889</v>
+      </c>
+      <c r="F3529">
+        <v>32.86</v>
+      </c>
+      <c r="G3529">
+        <v>67.33</v>
+      </c>
+      <c r="H3529">
+        <v>81.599999999999994</v>
+      </c>
+    </row>
+    <row r="3530" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3530" s="2">
+        <v>46057</v>
+      </c>
+      <c r="B3530">
+        <v>225.43</v>
+      </c>
+      <c r="C3530">
+        <v>618.12</v>
+      </c>
+      <c r="D3530">
+        <v>19.75</v>
+      </c>
+      <c r="E3530">
+        <v>2.8620000000000001</v>
+      </c>
+      <c r="F3530">
+        <v>33.500999999999998</v>
+      </c>
+      <c r="G3530">
+        <v>69.459999999999994</v>
+      </c>
+      <c r="H3530">
+        <v>81.430000000000007</v>
+      </c>
+    </row>
+    <row r="3531" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3531" s="2">
+        <v>46058</v>
+      </c>
+      <c r="B3531">
+        <v>225.65</v>
+      </c>
+      <c r="C3531">
+        <v>611.65</v>
+      </c>
+      <c r="D3531">
+        <v>21.1</v>
+      </c>
+      <c r="E3531">
+        <v>2.8433999999999999</v>
+      </c>
+      <c r="F3531">
+        <v>33.734999999999999</v>
+      </c>
+      <c r="G3531">
+        <v>67.55</v>
+      </c>
+      <c r="H3531">
+        <v>76.81</v>
+      </c>
+    </row>
+    <row r="3532" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3532" s="2">
+        <v>46059</v>
+      </c>
+      <c r="B3532">
+        <v>223.53</v>
+      </c>
+      <c r="C3532">
+        <v>617.12</v>
+      </c>
+      <c r="D3532">
+        <v>19.850000000000001</v>
+      </c>
+      <c r="E3532">
+        <v>2.8475999999999999</v>
+      </c>
+      <c r="F3532">
+        <v>35.694000000000003</v>
+      </c>
+      <c r="G3532">
+        <v>68.05</v>
+      </c>
+      <c r="H3532">
+        <v>77.319999999999993</v>
+      </c>
+    </row>
+    <row r="3533" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3533" s="2">
+        <v>46062</v>
+      </c>
+      <c r="B3533">
+        <v>225.77</v>
+      </c>
+      <c r="C3533">
+        <v>621.41</v>
+      </c>
+      <c r="D3533">
+        <v>18.7</v>
+      </c>
+      <c r="E3533">
+        <v>2.8393999999999999</v>
+      </c>
+      <c r="F3533">
+        <v>33.496000000000002</v>
+      </c>
+      <c r="G3533">
+        <v>69.040000000000006</v>
+      </c>
+      <c r="H3533">
+        <v>79.930000000000007</v>
+      </c>
+    </row>
+    <row r="3534" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3534" s="2">
+        <v>46063</v>
+      </c>
+      <c r="B3534">
+        <v>226.99</v>
+      </c>
+      <c r="C3534">
+        <v>620.97</v>
+      </c>
+      <c r="D3534">
+        <v>18.7</v>
+      </c>
+      <c r="E3534">
+        <v>2.8039999999999998</v>
+      </c>
+      <c r="F3534">
+        <v>31.846</v>
+      </c>
+      <c r="G3534">
+        <v>68.8</v>
+      </c>
+      <c r="H3534">
+        <v>77.45</v>
+      </c>
+    </row>
+    <row r="3535" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3535" s="2">
+        <v>46064</v>
+      </c>
+      <c r="B3535">
+        <v>226.81</v>
+      </c>
+      <c r="C3535">
+        <v>621.58000000000004</v>
+      </c>
+      <c r="D3535">
+        <v>18.75</v>
+      </c>
+      <c r="E3535">
+        <v>2.7959999999999998</v>
+      </c>
+      <c r="F3535">
+        <v>32.167000000000002</v>
+      </c>
+      <c r="G3535">
+        <v>69.400000000000006</v>
+      </c>
+      <c r="H3535">
+        <v>77.06</v>
+      </c>
+    </row>
+    <row r="3536" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3536" s="2">
+        <v>46065</v>
+      </c>
+      <c r="B3536">
+        <v>227.78</v>
+      </c>
+      <c r="C3536">
+        <v>618.52</v>
+      </c>
+      <c r="D3536">
+        <v>20.3</v>
+      </c>
+      <c r="E3536">
+        <v>2.7770000000000001</v>
+      </c>
+      <c r="F3536">
+        <v>32.994</v>
+      </c>
+      <c r="G3536">
+        <v>67.52</v>
+      </c>
+      <c r="H3536">
+        <v>71.260000000000005</v>
+      </c>
+    </row>
+    <row r="3537" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3537" s="2">
+        <v>46066</v>
+      </c>
+      <c r="B3537">
+        <v>225.96</v>
+      </c>
+      <c r="C3537">
+        <v>617.70000000000005</v>
+      </c>
+      <c r="D3537">
+        <v>20.25</v>
+      </c>
+      <c r="E3537">
+        <v>2.7572999999999999</v>
+      </c>
+      <c r="F3537">
+        <v>32.5</v>
+      </c>
+      <c r="G3537">
+        <v>67.75</v>
+      </c>
+      <c r="H3537">
+        <v>69.45</v>
+      </c>
+    </row>
+    <row r="3538" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3538" s="2">
+        <v>46069</v>
+      </c>
+      <c r="B3538">
+        <v>225.83</v>
+      </c>
+      <c r="C3538">
+        <v>618.52</v>
+      </c>
+      <c r="D3538">
+        <v>20.25</v>
+      </c>
+      <c r="E3538">
+        <v>2.7555999999999998</v>
+      </c>
+      <c r="F3538">
+        <v>30.754999999999999</v>
+      </c>
+      <c r="G3538">
+        <v>67.97</v>
+      </c>
+      <c r="H3538">
+        <v>67.97</v>
+      </c>
+    </row>
+    <row r="3539" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3539" s="2">
+        <v>46070</v>
+      </c>
+      <c r="B3539">
+        <v>225.19</v>
+      </c>
+      <c r="C3539">
+        <v>621.29</v>
+      </c>
+      <c r="D3539">
+        <v>19.55</v>
+      </c>
+      <c r="E3539">
+        <v>2.742</v>
+      </c>
+      <c r="F3539">
+        <v>29.821999999999999</v>
+      </c>
+      <c r="G3539">
+        <v>66.87</v>
+      </c>
+      <c r="H3539">
+        <v>68.88</v>
+      </c>
+    </row>
+    <row r="3540" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3540" s="2">
+        <v>46071</v>
+      </c>
+      <c r="B3540">
+        <v>227.08</v>
+      </c>
+      <c r="C3540">
+        <v>628.69000000000005</v>
+      </c>
+      <c r="D3540">
+        <v>18.13</v>
+      </c>
+      <c r="E3540">
+        <v>2.7427999999999999</v>
+      </c>
+      <c r="F3540">
+        <v>31.481000000000002</v>
+      </c>
+      <c r="G3540">
+        <v>69.77</v>
+      </c>
+      <c r="H3540">
+        <v>70.349999999999994</v>
+      </c>
+    </row>
+    <row r="3541" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3541" s="2">
+        <v>46072</v>
+      </c>
+      <c r="B3541">
+        <v>228.98</v>
+      </c>
+      <c r="C3541">
+        <v>625.33000000000004</v>
+      </c>
+      <c r="D3541">
+        <v>20.3</v>
+      </c>
+      <c r="E3541">
+        <v>2.7450999999999999</v>
+      </c>
+      <c r="F3541">
+        <v>33.523000000000003</v>
+      </c>
+      <c r="G3541">
+        <v>71.27</v>
+      </c>
+      <c r="H3541">
+        <v>70.11</v>
+      </c>
+    </row>
+    <row r="3542" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3542" s="2">
+        <v>46073</v>
+      </c>
+      <c r="B3542">
+        <v>228.05</v>
+      </c>
+      <c r="C3542">
+        <v>630.55999999999995</v>
+      </c>
+      <c r="D3542">
+        <v>19.7</v>
+      </c>
+      <c r="E3542">
+        <v>2.7385000000000002</v>
+      </c>
+      <c r="F3542">
+        <v>32.029000000000003</v>
+      </c>
+      <c r="G3542">
+        <v>71.3</v>
+      </c>
+      <c r="H3542">
+        <v>72.540000000000006</v>
+      </c>
+    </row>
+    <row r="3543" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3543" s="2">
+        <v>46076</v>
+      </c>
+      <c r="B3543">
+        <v>229.36</v>
+      </c>
+      <c r="C3543">
+        <v>627.70000000000005</v>
+      </c>
+      <c r="D3543">
+        <v>20.100000000000001</v>
+      </c>
+      <c r="E3543">
+        <v>2.7153</v>
+      </c>
+      <c r="F3543">
+        <v>31.834</v>
+      </c>
+      <c r="G3543">
+        <v>71.489999999999995</v>
+      </c>
+      <c r="H3543">
+        <v>70.14</v>
+      </c>
+    </row>
+    <row r="3544" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3544" s="2">
+        <v>46077</v>
+      </c>
+      <c r="B3544">
+        <v>228.56</v>
+      </c>
+      <c r="C3544">
+        <v>629.14</v>
+      </c>
+      <c r="D3544">
+        <v>19.649999999999999</v>
+      </c>
+      <c r="E3544">
+        <v>2.7075999999999998</v>
+      </c>
+      <c r="F3544">
+        <v>30.890999999999998</v>
+      </c>
+      <c r="G3544">
+        <v>70.77</v>
+      </c>
+      <c r="H3544">
+        <v>69.42</v>
+      </c>
+    </row>
+    <row r="3545" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3545" s="2">
+        <v>46078</v>
+      </c>
+      <c r="B3545">
+        <v>229.67</v>
+      </c>
+      <c r="C3545">
+        <v>633.47</v>
+      </c>
+      <c r="D3545">
+        <v>19.149999999999999</v>
+      </c>
+      <c r="E3545">
+        <v>2.7090000000000001</v>
+      </c>
+      <c r="F3545">
+        <v>31.05</v>
+      </c>
+      <c r="G3545">
+        <v>70.849999999999994</v>
+      </c>
+      <c r="H3545">
+        <v>71.31</v>
+      </c>
+    </row>
+    <row r="3546" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3546" s="2">
+        <v>46079</v>
+      </c>
+      <c r="B3546">
+        <v>230.89</v>
+      </c>
+      <c r="C3546">
+        <v>633.17999999999995</v>
+      </c>
+      <c r="D3546">
+        <v>19.600000000000001</v>
+      </c>
+      <c r="E3546">
+        <v>2.6983999999999999</v>
+      </c>
+      <c r="F3546">
+        <v>32.223999999999997</v>
+      </c>
+      <c r="G3546">
+        <v>70.75</v>
+      </c>
+      <c r="H3546">
+        <v>69.7</v>
+      </c>
+    </row>
+    <row r="3547" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3547" s="2">
+        <v>46080</v>
+      </c>
+      <c r="B3547">
+        <v>230.64</v>
+      </c>
+      <c r="C3547">
+        <v>633.85</v>
+      </c>
+      <c r="D3547">
+        <v>20.100000000000001</v>
+      </c>
+      <c r="E3547">
+        <v>2.6526999999999998</v>
+      </c>
+      <c r="F3547">
+        <v>31.959</v>
+      </c>
+      <c r="G3547">
+        <v>72.48</v>
+      </c>
+      <c r="H3547">
+        <v>69.02</v>
+      </c>
+    </row>
+    <row r="3548" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3548" s="2">
+        <v>46083</v>
+      </c>
+      <c r="B3548">
+        <v>228.71</v>
+      </c>
+      <c r="C3548">
+        <v>623.63</v>
+      </c>
+      <c r="D3548">
+        <v>21.3</v>
+      </c>
+      <c r="E3548">
+        <v>2.7081</v>
+      </c>
+      <c r="F3548">
+        <v>44.506</v>
+      </c>
+      <c r="G3548">
+        <v>77.739999999999995</v>
+      </c>
+      <c r="H3548">
+        <v>69.3</v>
+      </c>
+    </row>
+    <row r="3549" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3549" s="2">
+        <v>46084</v>
+      </c>
+      <c r="B3549">
+        <v>225.13</v>
+      </c>
+      <c r="C3549">
+        <v>604.44000000000005</v>
+      </c>
+      <c r="D3549">
+        <v>24.85</v>
+      </c>
+      <c r="E3549">
+        <v>2.7751999999999999</v>
+      </c>
+      <c r="F3549">
+        <v>54.29</v>
+      </c>
+      <c r="G3549">
+        <v>81.400000000000006</v>
+      </c>
+      <c r="H3549">
+        <v>71.98</v>
+      </c>
+    </row>
+    <row r="3550" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3550" s="2">
+        <v>46085</v>
+      </c>
+      <c r="B3550">
+        <v>219.64</v>
+      </c>
+      <c r="C3550">
+        <v>612.71</v>
+      </c>
+      <c r="D3550">
+        <v>22.4</v>
+      </c>
+      <c r="E3550">
+        <v>2.7458999999999998</v>
+      </c>
+      <c r="F3550">
+        <v>48.767000000000003</v>
+      </c>
+      <c r="G3550">
+        <v>81.400000000000006</v>
+      </c>
+      <c r="H3550">
+        <v>69.459999999999994</v>
+      </c>
+    </row>
+    <row r="3551" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3551" s="2">
+        <v>46086</v>
+      </c>
+      <c r="B3551">
+        <v>222.39</v>
+      </c>
+      <c r="C3551">
+        <v>604.83000000000004</v>
+      </c>
+      <c r="D3551">
+        <v>25.75</v>
+      </c>
+      <c r="E3551">
+        <v>2.8534999999999999</v>
+      </c>
+      <c r="F3551">
+        <v>50.731000000000002</v>
+      </c>
+      <c r="G3551">
+        <v>85.41</v>
+      </c>
+      <c r="H3551">
+        <v>69.02</v>
+      </c>
+    </row>
+    <row r="3552" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3552" s="2">
+        <v>46087</v>
+      </c>
+      <c r="B3552">
+        <v>220.44</v>
+      </c>
+      <c r="C3552">
+        <v>598.69000000000005</v>
+      </c>
+      <c r="D3552">
+        <v>28.4</v>
+      </c>
+      <c r="E3552">
+        <v>2.8643000000000001</v>
+      </c>
+      <c r="F3552">
+        <v>53.384999999999998</v>
+      </c>
+      <c r="G3552">
+        <v>92.69</v>
+      </c>
+      <c r="H3552">
+        <v>69.23</v>
+      </c>
+    </row>
+    <row r="3553" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3553" s="2">
+        <v>46090</v>
+      </c>
+      <c r="B3553">
+        <v>214.75</v>
+      </c>
+      <c r="C3553">
+        <v>594.91999999999996</v>
+      </c>
+      <c r="D3553">
+        <v>28.2</v>
+      </c>
+      <c r="E3553">
+        <v>2.8649</v>
+      </c>
+      <c r="F3553">
+        <v>56.453000000000003</v>
+      </c>
+      <c r="G3553">
+        <v>98.96</v>
+      </c>
+      <c r="H3553">
+        <v>69.540000000000006</v>
+      </c>
+    </row>
+    <row r="3554" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3554" s="2">
+        <v>46091</v>
+      </c>
+      <c r="B3554">
+        <v>216.32</v>
+      </c>
+      <c r="C3554">
+        <v>606.12</v>
+      </c>
+      <c r="D3554">
+        <v>25.45</v>
+      </c>
+      <c r="E3554">
+        <v>2.8532999999999999</v>
+      </c>
+      <c r="F3554">
+        <v>47.393000000000001</v>
+      </c>
+      <c r="G3554">
+        <v>87.8</v>
+      </c>
+      <c r="H3554">
+        <v>71.540000000000006</v>
+      </c>
+    </row>
+    <row r="3555" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3555" s="2">
+        <v>46092</v>
+      </c>
+      <c r="B3555">
+        <v>218.58</v>
+      </c>
+      <c r="C3555">
+        <v>602.54</v>
+      </c>
+      <c r="D3555">
+        <v>28.2</v>
+      </c>
+      <c r="E3555">
+        <v>2.9318</v>
+      </c>
+      <c r="F3555">
+        <v>49.988999999999997</v>
+      </c>
+      <c r="G3555">
+        <v>91.98</v>
+      </c>
+      <c r="H3555">
+        <v>70.47</v>
+      </c>
+    </row>
+    <row r="3556" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3556" s="2">
+        <v>46093</v>
+      </c>
+      <c r="B3556">
+        <v>217.18</v>
+      </c>
+      <c r="C3556">
+        <v>598.86</v>
+      </c>
+      <c r="D3556">
+        <v>29.05</v>
+      </c>
+      <c r="E3556">
+        <v>2.9378000000000002</v>
+      </c>
+      <c r="F3556">
+        <v>50.87</v>
+      </c>
+      <c r="G3556">
+        <v>100.46</v>
+      </c>
+      <c r="H3556">
+        <v>67.400000000000006</v>
+      </c>
+    </row>
+    <row r="3557" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3557" s="2">
+        <v>46094</v>
+      </c>
+      <c r="B3557">
+        <v>215.2</v>
+      </c>
+      <c r="C3557">
+        <v>595.85</v>
+      </c>
+      <c r="D3557">
+        <v>28.5</v>
+      </c>
+      <c r="E3557">
+        <v>2.9767999999999999</v>
+      </c>
+      <c r="F3557">
+        <v>50.115000000000002</v>
+      </c>
+      <c r="G3557">
+        <v>103.14</v>
+      </c>
+      <c r="H3557">
+        <v>67.83</v>
+      </c>
+    </row>
+    <row r="3558" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3558" s="2">
+        <v>46097</v>
+      </c>
+      <c r="B3558">
+        <v>214.86</v>
+      </c>
+      <c r="C3558">
+        <v>598.47</v>
+      </c>
+      <c r="D3558">
+        <v>27.2</v>
+      </c>
+      <c r="E3558">
+        <v>2.9487999999999999</v>
+      </c>
+      <c r="F3558">
+        <v>50.887</v>
+      </c>
+      <c r="G3558">
+        <v>96.04</v>
+      </c>
+      <c r="H3558">
+        <v>67.650000000000006</v>
+      </c>
+    </row>
+    <row r="3559" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3559" s="2">
+        <v>46098</v>
+      </c>
+      <c r="B3559">
+        <v>215.54</v>
+      </c>
+      <c r="C3559">
+        <v>602.45000000000005</v>
+      </c>
+      <c r="D3559">
+        <v>25.85</v>
+      </c>
+      <c r="E3559">
+        <v>2.9028</v>
+      </c>
+      <c r="F3559">
+        <v>51.558999999999997</v>
+      </c>
+      <c r="G3559">
+        <v>99.39</v>
+      </c>
+      <c r="H3559">
+        <v>65.81</v>
+      </c>
+    </row>
+    <row r="3560" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3560" s="2">
+        <v>46099</v>
+      </c>
+      <c r="B3560">
+        <v>217.42</v>
+      </c>
+      <c r="C3560">
+        <v>597.92999999999995</v>
+      </c>
+      <c r="D3560">
+        <v>24.78</v>
+      </c>
+      <c r="E3560">
+        <v>2.9424999999999999</v>
+      </c>
+      <c r="F3560">
+        <v>54.661999999999999</v>
+      </c>
+      <c r="G3560">
+        <v>102.92</v>
+      </c>
+      <c r="H3560">
+        <v>65.040000000000006</v>
+      </c>
+    </row>
+    <row r="3561" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3561" s="2">
+        <v>46100</v>
+      </c>
+      <c r="B3561">
+        <v>213.56</v>
+      </c>
+      <c r="C3561">
+        <v>583.64</v>
+      </c>
+      <c r="D3561">
+        <v>27.7</v>
+      </c>
+      <c r="E3561">
+        <v>2.9523999999999999</v>
+      </c>
+      <c r="F3561">
+        <v>61.851999999999997</v>
+      </c>
+      <c r="G3561">
+        <v>103.78</v>
+      </c>
+      <c r="H3561">
+        <v>62.8</v>
+      </c>
+    </row>
+    <row r="3562" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3562" s="2">
+        <v>46101</v>
+      </c>
+      <c r="B3562">
+        <v>210.35</v>
+      </c>
+      <c r="C3562">
+        <v>573.28</v>
+      </c>
+      <c r="D3562">
+        <v>28.6</v>
+      </c>
+      <c r="E3562">
+        <v>3.0381</v>
+      </c>
+      <c r="F3562">
+        <v>59.255000000000003</v>
+      </c>
+      <c r="G3562">
+        <v>106.41</v>
+      </c>
+      <c r="H3562">
+        <v>66.73</v>
+      </c>
+    </row>
+    <row r="3563" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3563" s="2">
+        <v>46104</v>
+      </c>
+      <c r="B3563">
+        <v>204.19</v>
+      </c>
+      <c r="C3563">
+        <v>576.78</v>
+      </c>
+      <c r="D3563">
+        <v>28.1</v>
+      </c>
+      <c r="E3563">
+        <v>3.0186000000000002</v>
+      </c>
+      <c r="F3563">
+        <v>56.683</v>
+      </c>
+      <c r="G3563">
+        <v>95.92</v>
+      </c>
+      <c r="H3563">
+        <v>68.31</v>
+      </c>
+    </row>
+    <row r="3564" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3564" s="2">
+        <v>46105</v>
+      </c>
+      <c r="B3564">
+        <v>207.82</v>
+      </c>
+      <c r="C3564">
+        <v>579.28</v>
+      </c>
+      <c r="D3564">
+        <v>28.45</v>
+      </c>
+      <c r="E3564">
+        <v>3.0135000000000001</v>
+      </c>
+      <c r="F3564">
+        <v>54.040999999999997</v>
+      </c>
+      <c r="G3564">
+        <v>100.23</v>
+      </c>
+      <c r="H3564">
+        <v>70.209999999999994</v>
+      </c>
+    </row>
+    <row r="3565" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3565" s="2">
+        <v>46106</v>
+      </c>
+      <c r="B3565">
+        <v>209.21</v>
+      </c>
+      <c r="C3565">
+        <v>587.49</v>
+      </c>
+      <c r="D3565">
+        <v>27.65</v>
+      </c>
+      <c r="E3565">
+        <v>2.9535</v>
+      </c>
+      <c r="F3565">
+        <v>52.816000000000003</v>
+      </c>
+      <c r="G3565">
+        <v>102.22</v>
+      </c>
+      <c r="H3565">
+        <v>69.739999999999995</v>
+      </c>
+    </row>
+    <row r="3566" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3566" s="2">
+        <v>46107</v>
+      </c>
+      <c r="B3566">
+        <v>210.41</v>
+      </c>
+      <c r="C3566">
+        <v>580.84</v>
+      </c>
+      <c r="D3566">
+        <v>28.9</v>
+      </c>
+      <c r="E3566">
+        <v>3.0630999999999999</v>
+      </c>
+      <c r="F3566">
+        <v>55.218000000000004</v>
+      </c>
+      <c r="G3566">
+        <v>108.01</v>
+      </c>
+      <c r="H3566">
+        <v>70.62</v>
+      </c>
+    </row>
+    <row r="3567" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3567" s="2">
+        <v>46108</v>
+      </c>
+      <c r="B3567">
+        <v>208.7</v>
+      </c>
+      <c r="C3567">
+        <v>575.29999999999995</v>
+      </c>
+      <c r="D3567">
+        <v>30.15</v>
+      </c>
+      <c r="E3567">
+        <v>3.0985</v>
+      </c>
+      <c r="F3567">
+        <v>54.177</v>
+      </c>
+      <c r="G3567">
+        <v>112.57</v>
+      </c>
+      <c r="H3567">
+        <v>70.63</v>
+      </c>
+    </row>
+    <row r="3568" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3568" s="2">
+        <v>46111</v>
+      </c>
+      <c r="B3568">
+        <v>206.35</v>
+      </c>
+      <c r="C3568">
+        <v>580.73</v>
+      </c>
+      <c r="D3568">
+        <v>29.9</v>
+      </c>
+      <c r="E3568">
+        <v>3.0390000000000001</v>
+      </c>
+      <c r="F3568">
+        <v>54.814</v>
+      </c>
+      <c r="G3568">
+        <v>112.78</v>
+      </c>
+      <c r="H3568">
+        <v>71.13</v>
+      </c>
+    </row>
+    <row r="3569" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3569" s="2">
+        <v>46112</v>
+      </c>
+      <c r="B3569">
+        <v>208.62</v>
+      </c>
+      <c r="C3569">
+        <v>583.14</v>
+      </c>
+      <c r="D3569">
+        <v>28.3</v>
+      </c>
+      <c r="E3569">
+        <v>3.0076000000000001</v>
+      </c>
+      <c r="F3569">
+        <v>50.756999999999998</v>
+      </c>
+      <c r="G3569">
+        <v>118.35</v>
+      </c>
+      <c r="H3569">
+        <v>71.47</v>
+      </c>
+    </row>
+    <row r="3570" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3570" s="2">
+        <v>46113</v>
+      </c>
+      <c r="B3570">
+        <v>211.35</v>
+      </c>
+      <c r="C3570">
+        <v>597.69000000000005</v>
+      </c>
+      <c r="D3570">
+        <v>25.75</v>
+      </c>
+      <c r="E3570">
+        <v>2.9962</v>
+      </c>
+      <c r="F3570">
+        <v>47.51</v>
+      </c>
+      <c r="G3570">
+        <v>101.16</v>
+      </c>
+      <c r="H3570">
+        <v>73.599999999999994</v>
+      </c>
+    </row>
+    <row r="3571" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3571" s="2">
+        <v>46114</v>
+      </c>
+      <c r="B3571">
+        <v>213.27</v>
+      </c>
+      <c r="C3571">
+        <v>596.63</v>
+      </c>
+      <c r="D3571">
+        <v>27.45</v>
+      </c>
+      <c r="E3571">
+        <v>2.9954999999999998</v>
+      </c>
+      <c r="F3571">
+        <v>50.043999999999997</v>
+      </c>
+      <c r="G3571">
+        <v>109.03</v>
+      </c>
+      <c r="H3571">
+        <v>70.67</v>
+      </c>
+    </row>
+    <row r="3572" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3572" s="2">
+        <v>46119</v>
+      </c>
+      <c r="B3572">
+        <v>214.81</v>
+      </c>
+      <c r="C3572">
+        <v>590.59</v>
+      </c>
+      <c r="D3572">
+        <v>28.85</v>
+      </c>
+      <c r="E3572">
+        <v>3.0830000000000002</v>
+      </c>
+      <c r="F3572">
+        <v>53.247</v>
+      </c>
+      <c r="G3572">
+        <v>109.27</v>
+      </c>
+      <c r="H3572">
+        <v>70.48</v>
+      </c>
+    </row>
+    <row r="3573" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3573" s="2">
+        <v>46120</v>
+      </c>
+      <c r="B3573">
+        <v>214.16</v>
+      </c>
+      <c r="C3573">
+        <v>613.5</v>
+      </c>
+      <c r="D3573">
+        <v>23.95</v>
+      </c>
+      <c r="E3573">
+        <v>2.9422999999999999</v>
+      </c>
+      <c r="F3573">
+        <v>45.301000000000002</v>
+      </c>
+      <c r="G3573">
+        <v>94.75</v>
+      </c>
+      <c r="H3573">
+        <v>70.72</v>
+      </c>
+    </row>
+    <row r="3574" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3574" s="2">
+        <v>46121</v>
+      </c>
+      <c r="B3574">
+        <v>220.82</v>
+      </c>
+      <c r="C3574">
+        <v>612.59</v>
+      </c>
+      <c r="D3574">
+        <v>23.45</v>
+      </c>
+      <c r="E3574">
+        <v>3.0101</v>
+      </c>
+      <c r="F3574">
+        <v>46.174999999999997</v>
+      </c>
+      <c r="G3574">
+        <v>95.92</v>
+      </c>
+      <c r="H3574">
+        <v>72.73</v>
+      </c>
+    </row>
+    <row r="3575" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3575" s="2">
+        <v>46122</v>
+      </c>
+      <c r="B3575">
+        <v>220.82</v>
+      </c>
+      <c r="C3575">
+        <v>614.84</v>
+      </c>
+      <c r="D3575">
+        <v>22.1</v>
+      </c>
+      <c r="E3575">
+        <v>3.0480999999999998</v>
+      </c>
+      <c r="F3575">
+        <v>43.637999999999998</v>
+      </c>
+      <c r="G3575">
+        <v>95.2</v>
+      </c>
+      <c r="H3575">
+        <v>71.84</v>
+      </c>
+    </row>
+    <row r="3576" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3576" s="2">
+        <v>46125</v>
+      </c>
+      <c r="B3576">
+        <v>220.96</v>
+      </c>
+      <c r="C3576">
+        <v>613.88</v>
+      </c>
+      <c r="D3576">
+        <v>22.6</v>
+      </c>
+      <c r="E3576">
+        <v>3.0901999999999998</v>
+      </c>
+      <c r="F3576">
+        <v>46.412999999999997</v>
+      </c>
+      <c r="G3576">
+        <v>99.36</v>
+      </c>
+      <c r="H3576">
+        <v>71.599999999999994</v>
+      </c>
+    </row>
+    <row r="3577" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3577" s="2">
+        <v>46126</v>
+      </c>
+      <c r="B3577">
+        <v>221.72</v>
+      </c>
+      <c r="C3577">
+        <v>619.95000000000005</v>
+      </c>
+      <c r="D3577">
+        <v>20.05</v>
+      </c>
+      <c r="E3577">
+        <v>3.0297000000000001</v>
+      </c>
+      <c r="F3577">
+        <v>43.365000000000002</v>
+      </c>
+      <c r="G3577">
+        <v>94.79</v>
+      </c>
+      <c r="H3577">
+        <v>73.86</v>
+      </c>
+    </row>
+    <row r="3578" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3578" s="2">
+        <v>46127</v>
+      </c>
+      <c r="B3578">
+        <v>224.1</v>
+      </c>
+      <c r="C3578">
+        <v>617.27</v>
+      </c>
+      <c r="D3578">
+        <v>21.02</v>
+      </c>
+      <c r="E3578">
+        <v>3.0474000000000001</v>
+      </c>
+      <c r="F3578">
+        <v>41.399000000000001</v>
+      </c>
+      <c r="G3578">
+        <v>94.93</v>
+      </c>
+      <c r="H3578">
+        <v>73.150000000000006</v>
+      </c>
+    </row>
+    <row r="3579" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3579" s="2">
+        <v>46128</v>
+      </c>
+      <c r="B3579">
+        <v>223.3</v>
+      </c>
+      <c r="C3579">
+        <v>616.95000000000005</v>
+      </c>
+      <c r="D3579">
+        <v>21.25</v>
+      </c>
+      <c r="E3579">
+        <v>3.0318999999999998</v>
+      </c>
+      <c r="F3579">
+        <v>42.421999999999997</v>
+      </c>
+      <c r="G3579">
+        <v>99.39</v>
+      </c>
+      <c r="H3579">
+        <v>73.989999999999995</v>
+      </c>
+    </row>
+    <row r="3580" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3580" s="2">
+        <v>46129</v>
+      </c>
+      <c r="B3580">
+        <v>222.64</v>
+      </c>
+      <c r="C3580">
+        <v>626.58000000000004</v>
+      </c>
+      <c r="D3580">
+        <v>20.2</v>
+      </c>
+      <c r="E3580">
+        <v>2.9651000000000001</v>
+      </c>
+      <c r="F3580">
+        <v>38.768999999999998</v>
+      </c>
+      <c r="G3580">
+        <v>90.38</v>
+      </c>
+      <c r="H3580">
+        <v>76.47</v>
+      </c>
+    </row>
+    <row r="3581" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3581" s="2">
+        <v>46132</v>
+      </c>
+      <c r="B3581">
+        <v>225.56</v>
+      </c>
+      <c r="C3581">
+        <v>621.46</v>
+      </c>
+      <c r="D3581">
+        <v>21.65</v>
+      </c>
+      <c r="E3581">
+        <v>2.9765000000000001</v>
+      </c>
+      <c r="F3581">
+        <v>40.292000000000002</v>
+      </c>
+      <c r="G3581">
+        <v>90.43</v>
+      </c>
+      <c r="H3581">
+        <v>75.14</v>
+      </c>
+    </row>
+    <row r="3582" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3582" s="2">
+        <v>46133</v>
+      </c>
+      <c r="B3582">
+        <v>225.43</v>
+      </c>
+      <c r="C3582">
+        <v>616.03</v>
+      </c>
+      <c r="D3582">
+        <v>22.05</v>
+      </c>
+      <c r="E3582">
+        <v>3.0108000000000001</v>
+      </c>
+      <c r="F3582">
+        <v>41.930999999999997</v>
+      </c>
+      <c r="G3582">
+        <v>93.24</v>
+      </c>
+      <c r="H3582">
+        <v>74.709999999999994</v>
+      </c>
+    </row>
+    <row r="3583" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3583" s="2">
+        <v>46134</v>
+      </c>
+      <c r="B3583">
+        <v>223.89</v>
+      </c>
+      <c r="C3583">
+        <v>613.88</v>
+      </c>
+      <c r="D3583">
+        <v>22</v>
+      </c>
+      <c r="E3583">
+        <v>3.0005000000000002</v>
+      </c>
+      <c r="F3583">
+        <v>43.552</v>
+      </c>
+      <c r="G3583">
+        <v>96.18</v>
+      </c>
+      <c r="H3583">
+        <v>73.42</v>
+      </c>
+    </row>
+    <row r="3584" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3584" s="2">
+        <v>46135</v>
+      </c>
+      <c r="B3584">
+        <v>222.02</v>
+      </c>
+      <c r="C3584">
+        <v>614.20000000000005</v>
+      </c>
+      <c r="D3584">
+        <v>22</v>
+      </c>
+      <c r="E3584">
+        <v>3.0042</v>
+      </c>
+      <c r="F3584">
+        <v>44.496000000000002</v>
+      </c>
+      <c r="G3584">
+        <v>99.35</v>
+      </c>
+      <c r="H3584">
+        <v>73.849999999999994</v>
+      </c>
+    </row>
+    <row r="3585" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3585" s="2">
+        <v>46136</v>
+      </c>
+      <c r="B3585">
+        <v>221.88</v>
+      </c>
+      <c r="C3585">
+        <v>610.65</v>
+      </c>
+      <c r="D3585">
+        <v>22.25</v>
+      </c>
+      <c r="E3585">
+        <v>3.0068000000000001</v>
+      </c>
+      <c r="F3585">
+        <v>44.860999999999997</v>
+      </c>
+      <c r="G3585">
+        <v>105.33</v>
+      </c>
+      <c r="H3585">
+        <v>73.92</v>
+      </c>
+    </row>
+    <row r="3586" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3586" s="2">
+        <v>46139</v>
+      </c>
+      <c r="B3586">
+        <v>221.53</v>
+      </c>
+      <c r="C3586">
+        <v>608.84</v>
+      </c>
+      <c r="D3586">
+        <v>22.55</v>
+      </c>
+      <c r="E3586">
+        <v>3.036</v>
+      </c>
+      <c r="F3586">
+        <v>44.646000000000001</v>
+      </c>
+      <c r="G3586">
+        <v>108.23</v>
+      </c>
+      <c r="H3586">
+        <v>73.75</v>
+      </c>
+    </row>
+    <row r="3587" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3587" s="2">
+        <v>46140</v>
+      </c>
+      <c r="B3587">
+        <v>220.57</v>
+      </c>
+      <c r="C3587">
+        <v>606.58000000000004</v>
+      </c>
+      <c r="D3587">
+        <v>22.3</v>
+      </c>
+      <c r="E3587">
+        <v>3.0613000000000001</v>
+      </c>
+      <c r="F3587">
+        <v>43.594000000000001</v>
+      </c>
+      <c r="G3587">
+        <v>111.26</v>
+      </c>
+      <c r="H3587">
+        <v>74.099999999999994</v>
+      </c>
+    </row>
+    <row r="3588" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3588" s="2">
+        <v>46141</v>
+      </c>
+      <c r="B3588">
+        <v>220.04</v>
+      </c>
+      <c r="C3588">
+        <v>602.96</v>
+      </c>
+      <c r="D3588">
+        <v>22.4</v>
+      </c>
+      <c r="E3588">
+        <v>3.0964</v>
+      </c>
+      <c r="F3588">
+        <v>46.853000000000002</v>
+      </c>
+      <c r="G3588">
+        <v>118.03</v>
+      </c>
+      <c r="H3588">
+        <v>72.19</v>
+      </c>
+    </row>
+    <row r="3589" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3589" s="2">
+        <v>46142</v>
+      </c>
+      <c r="B3589">
+        <v>217.31</v>
+      </c>
+      <c r="C3589">
+        <v>611.28</v>
+      </c>
+      <c r="D3589">
+        <v>21.65</v>
+      </c>
+      <c r="E3589">
+        <v>3.0297000000000001</v>
+      </c>
+      <c r="F3589">
+        <v>45.987000000000002</v>
+      </c>
+      <c r="G3589">
+        <v>114.01</v>
+      </c>
+      <c r="H3589">
+        <v>72.78</v>
+      </c>
+    </row>
+    <row r="3590" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3590" s="2">
+        <v>46146</v>
+      </c>
+      <c r="B3590">
+        <v>221.46</v>
+      </c>
+      <c r="C3590">
+        <v>605.51</v>
+      </c>
+      <c r="D3590">
+        <v>22.6</v>
+      </c>
+      <c r="E3590">
+        <v>3.0828000000000002</v>
+      </c>
+      <c r="F3590">
+        <v>48.143000000000001</v>
+      </c>
+      <c r="G3590">
+        <v>114.44</v>
+      </c>
+      <c r="H3590">
+        <v>72.02</v>
+      </c>
+    </row>
+    <row r="3591" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3591" s="2">
+        <v>46147</v>
+      </c>
+      <c r="B3591">
+        <v>218.63</v>
+      </c>
+      <c r="C3591">
+        <v>609.72</v>
+      </c>
+      <c r="D3591">
+        <v>22.05</v>
+      </c>
+      <c r="E3591">
+        <v>3.0663</v>
+      </c>
+      <c r="F3591">
+        <v>46.926000000000002</v>
+      </c>
+      <c r="G3591">
+        <v>109.87</v>
+      </c>
+      <c r="H3591">
+        <v>74.66</v>
+      </c>
+    </row>
+    <row r="3592" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3592" s="2">
+        <v>46148</v>
+      </c>
+      <c r="B3592">
+        <v>221.23</v>
+      </c>
+      <c r="C3592">
+        <v>623.25</v>
+      </c>
+      <c r="D3592">
+        <v>20.65</v>
+      </c>
+      <c r="E3592">
+        <v>2.9943</v>
+      </c>
+      <c r="F3592">
+        <v>43.902000000000001</v>
+      </c>
+      <c r="G3592">
+        <v>101.27</v>
+      </c>
+      <c r="H3592">
+        <v>75.02</v>
+      </c>
+    </row>
+    <row r="3593" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3593" s="2">
+        <v>46149</v>
+      </c>
+      <c r="B3593">
+        <v>225.9</v>
+      </c>
+      <c r="C3593">
+        <v>616.41999999999996</v>
+      </c>
+      <c r="D3593">
+        <v>21.2</v>
+      </c>
+      <c r="E3593">
+        <v>2.9971999999999999</v>
+      </c>
+      <c r="F3593">
+        <v>43.561</v>
+      </c>
+      <c r="G3593">
+        <v>100.06</v>
+      </c>
+      <c r="H3593">
+        <v>74.11</v>
+      </c>
+    </row>
+    <row r="3594" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3594" s="2">
+        <v>46150</v>
+      </c>
+      <c r="B3594">
+        <v>222.76</v>
+      </c>
+      <c r="C3594">
+        <v>612.14</v>
+      </c>
+      <c r="D3594">
+        <v>21.45</v>
+      </c>
+      <c r="E3594">
+        <v>3.0047000000000001</v>
+      </c>
+      <c r="F3594">
+        <v>44.143000000000001</v>
+      </c>
+      <c r="G3594">
+        <v>101.29</v>
+      </c>
+      <c r="H3594">
+        <v>74.150000000000006</v>
+      </c>
+    </row>
+    <row r="3595" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3595" s="2">
+        <v>46153</v>
+      </c>
+      <c r="B3595">
+        <v>222.16</v>
+      </c>
+      <c r="C3595">
+        <v>612.79</v>
+      </c>
+      <c r="D3595">
+        <v>21.45</v>
+      </c>
+      <c r="E3595">
+        <v>3.0432999999999999</v>
+      </c>
+      <c r="F3595">
+        <v>46.232999999999997</v>
+      </c>
+      <c r="G3595">
+        <v>104.21</v>
+      </c>
+      <c r="H3595">
+        <v>76.150000000000006</v>
+      </c>
+    </row>
+    <row r="3596" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3596" s="2">
+        <v>46154</v>
+      </c>
+      <c r="B3596">
+        <v>220.79</v>
+      </c>
+      <c r="C3596">
+        <v>606.63</v>
+      </c>
+      <c r="D3596">
+        <v>22.45</v>
+      </c>
+      <c r="E3596">
+        <v>3.0966</v>
+      </c>
+      <c r="F3596">
+        <v>46.683999999999997</v>
+      </c>
+      <c r="G3596">
+        <v>107.77</v>
+      </c>
+      <c r="H3596">
+        <v>74.77</v>
+      </c>
+    </row>
+    <row r="3597" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3597" s="2">
+        <v>46155</v>
+      </c>
+      <c r="B3597">
+        <v>220.49</v>
+      </c>
+      <c r="C3597">
+        <v>611.41999999999996</v>
+      </c>
+      <c r="D3597">
+        <v>21.5</v>
+      </c>
+      <c r="E3597">
+        <v>3.1097999999999999</v>
+      </c>
+      <c r="F3597">
+        <v>46.92</v>
+      </c>
+      <c r="G3597">
+        <v>105.63</v>
+      </c>
+      <c r="H3597">
+        <v>74.05</v>
+      </c>
+    </row>
+    <row r="3598" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3598" s="2">
+        <v>46156</v>
+      </c>
+      <c r="B3598">
+        <v>222.07</v>
+      </c>
+      <c r="C3598">
+        <v>616.04999999999995</v>
+      </c>
+      <c r="D3598">
+        <v>21.05</v>
+      </c>
+      <c r="E3598">
+        <v>3.0484</v>
+      </c>
+      <c r="F3598">
+        <v>47.655000000000001</v>
+      </c>
+      <c r="G3598">
+        <v>105.72</v>
+      </c>
+      <c r="H3598">
+        <v>74.069999999999993</v>
+      </c>
+    </row>
+    <row r="3599" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3599" s="2">
+        <v>46157</v>
+      </c>
+      <c r="B3599">
+        <v>222.68</v>
+      </c>
+      <c r="C3599">
+        <v>606.91999999999996</v>
+      </c>
+      <c r="D3599">
+        <v>21.5</v>
+      </c>
+      <c r="E3599">
+        <v>3.1535000000000002</v>
+      </c>
+      <c r="F3599">
+        <v>50.167000000000002</v>
+      </c>
+      <c r="G3599">
+        <v>109.26</v>
+      </c>
+      <c r="H3599">
+        <v>74.58</v>
+      </c>
+    </row>
+    <row r="3600" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3600" s="2">
+        <v>46160</v>
+      </c>
+      <c r="B3600">
+        <v>219.22</v>
+      </c>
+      <c r="C3600">
+        <v>610.16999999999996</v>
+      </c>
+      <c r="D3600">
+        <v>22.35</v>
+      </c>
+      <c r="E3600">
+        <v>3.1614</v>
+      </c>
+      <c r="F3600">
+        <v>50.25</v>
+      </c>
+      <c r="G3600">
+        <v>107.48</v>
+      </c>
+      <c r="H3600">
+        <v>74.53</v>
+      </c>
+    </row>
+    <row r="3601" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3601" s="2">
+        <v>46161</v>
+      </c>
+      <c r="B3601">
+        <v>221.17</v>
+      </c>
+      <c r="C3601">
+        <v>611.34</v>
+      </c>
+      <c r="D3601">
+        <v>22.45</v>
+      </c>
+      <c r="E3601">
+        <v>3.1884999999999999</v>
+      </c>
+      <c r="F3601">
+        <v>51.816000000000003</v>
+      </c>
+      <c r="G3601">
+        <v>106.71</v>
+      </c>
+      <c r="H3601">
+        <v>73.95</v>
+      </c>
+    </row>
+    <row r="3602" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3602" s="2">
+        <v>46162</v>
+      </c>
+      <c r="B3602">
+        <v>221.15</v>
+      </c>
+      <c r="C3602">
+        <v>620.29</v>
+      </c>
+      <c r="D3602">
+        <v>23.07</v>
+      </c>
+      <c r="E3602">
+        <v>3.0945</v>
+      </c>
+      <c r="F3602">
+        <v>49.424999999999997</v>
+      </c>
+      <c r="G3602">
+        <v>101.04</v>
+      </c>
+      <c r="H3602">
+        <v>74.37</v>
+      </c>
+    </row>
+    <row r="3603" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3603" s="2">
+        <v>46163</v>
+      </c>
+      <c r="B3603">
+        <v>224.45</v>
+      </c>
+      <c r="C3603">
+        <v>620.55999999999995</v>
+      </c>
+      <c r="D3603">
+        <v>21.85</v>
+      </c>
+      <c r="E3603">
+        <v>3.1012</v>
+      </c>
+      <c r="F3603">
+        <v>49.408000000000001</v>
+      </c>
+      <c r="G3603">
+        <v>99.5</v>
+      </c>
+      <c r="H3603">
+        <v>73.92</v>
+      </c>
+    </row>
+    <row r="3604" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3604" s="2">
+        <v>46164</v>
+      </c>
+      <c r="B3604">
+        <v>225.7</v>
+      </c>
+      <c r="C3604">
+        <v>625.12</v>
+      </c>
+      <c r="D3604">
+        <v>21.4</v>
+      </c>
+      <c r="E3604">
+        <v>3.0337999999999998</v>
+      </c>
+      <c r="F3604">
+        <v>48.683</v>
+      </c>
+      <c r="G3604">
+        <v>100.21</v>
+      </c>
+      <c r="H3604">
+        <v>75.900000000000006</v>
+      </c>
+    </row>
+    <row r="3605" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3605" s="2">
+        <v>46168</v>
+      </c>
+      <c r="B3605">
+        <v>229.22</v>
+      </c>
+      <c r="C3605">
+        <v>628.01</v>
+      </c>
+      <c r="D3605">
+        <v>20.5</v>
+      </c>
+      <c r="E3605">
+        <v>2.9836</v>
+      </c>
+      <c r="F3605">
+        <v>47.472000000000001</v>
+      </c>
+      <c r="G3605">
+        <v>99.58</v>
+      </c>
+      <c r="H3605">
+        <v>77.02</v>
+      </c>
+    </row>
+    <row r="3606" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3606" s="2">
+        <v>46169</v>
+      </c>
+      <c r="B3606">
+        <v>227.92</v>
+      </c>
+      <c r="C3606">
+        <v>628.17999999999995</v>
+      </c>
+      <c r="D3606">
+        <v>20.5</v>
+      </c>
+      <c r="E3606">
+        <v>2.9843000000000002</v>
+      </c>
+      <c r="F3606">
+        <v>46.412999999999997</v>
+      </c>
+      <c r="G3606">
+        <v>94.29</v>
+      </c>
+      <c r="H3606">
+        <v>77.69</v>
+      </c>
+    </row>
+    <row r="3607" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3607" s="2">
+        <v>46170</v>
+      </c>
+      <c r="B3607">
+        <v>227.63</v>
+      </c>
+      <c r="C3607">
+        <v>625.11</v>
+      </c>
+      <c r="D3607">
+        <v>20</v>
+      </c>
+      <c r="E3607">
+        <v>2.9596</v>
+      </c>
+      <c r="F3607">
+        <v>46.920999999999999</v>
+      </c>
+      <c r="G3607">
+        <v>93.71</v>
+      </c>
+      <c r="H3607">
+        <v>79.12</v>
+      </c>
+    </row>
+    <row r="3608" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3608" s="2">
+        <v>46171</v>
+      </c>
+      <c r="B3608">
+        <v>227.03</v>
+      </c>
+      <c r="C3608">
+        <v>626</v>
+      </c>
+      <c r="D3608">
+        <v>19.7</v>
+      </c>
+      <c r="E3608">
+        <v>2.9327999999999999</v>
+      </c>
+      <c r="F3608">
+        <v>46.000999999999998</v>
+      </c>
+      <c r="G3608">
+        <v>92.05</v>
+      </c>
+      <c r="H3608">
+        <v>79.59</v>
+      </c>
+    </row>
+    <row r="3609" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3609" s="2">
+        <v>46174</v>
+      </c>
+      <c r="B3609">
+        <v>226.91</v>
+      </c>
+      <c r="C3609">
+        <v>621.24</v>
+      </c>
+      <c r="D3609">
+        <v>20.25</v>
+      </c>
+      <c r="E3609">
+        <v>3.0129999999999999</v>
+      </c>
+      <c r="F3609">
+        <v>49.09</v>
+      </c>
+      <c r="G3609">
+        <v>94.98</v>
+      </c>
+      <c r="H3609">
+        <v>78.13</v>
+      </c>
+    </row>
+    <row r="3610" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3610" s="2">
+        <v>46175</v>
+      </c>
+      <c r="B3610">
+        <v>225.95</v>
+      </c>
+      <c r="C3610">
+        <v>625.34</v>
+      </c>
+      <c r="D3610">
+        <v>19.649999999999999</v>
+      </c>
+      <c r="E3610">
+        <v>2.9744000000000002</v>
+      </c>
+      <c r="F3610">
+        <v>47.606999999999999</v>
+      </c>
+      <c r="G3610">
+        <v>96</v>
+      </c>
+      <c r="H3610">
+        <v>78.45</v>
+      </c>
+    </row>
+    <row r="3611" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3611" s="2">
+        <v>46176</v>
+      </c>
+      <c r="B3611">
+        <v>226.89</v>
+      </c>
+      <c r="C3611">
+        <v>621.19000000000005</v>
+      </c>
+      <c r="D3611">
+        <v>19.75</v>
+      </c>
+      <c r="E3611">
+        <v>3.0367000000000002</v>
+      </c>
+      <c r="F3611">
+        <v>48.863999999999997</v>
+      </c>
+      <c r="G3611">
+        <v>97.81</v>
+      </c>
+      <c r="H3611">
+        <v>77.55</v>
+      </c>
+    </row>
+    <row r="3612" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3612" s="2">
+        <v>46177</v>
+      </c>
+      <c r="B3612">
+        <v>225.27</v>
+      </c>
+      <c r="C3612">
+        <v>624.45000000000005</v>
+      </c>
+      <c r="D3612">
+        <v>19.149999999999999</v>
+      </c>
+      <c r="E3612">
+        <v>3.0236999999999998</v>
+      </c>
+      <c r="F3612">
+        <v>48.752000000000002</v>
+      </c>
+      <c r="G3612">
+        <v>95.03</v>
+      </c>
+      <c r="H3612">
+        <v>76.03</v>
+      </c>
+    </row>
+    <row r="3613" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3613" s="2">
+        <v>46178</v>
+      </c>
+      <c r="B3613">
+        <v>226.77</v>
+      </c>
+      <c r="C3613">
+        <v>622.66</v>
+      </c>
+      <c r="D3613">
+        <v>19.45</v>
+      </c>
+      <c r="E3613">
+        <v>3.0375999999999999</v>
+      </c>
+      <c r="F3613">
+        <v>48.496000000000002</v>
+      </c>
+      <c r="G3613">
+        <v>93.09</v>
+      </c>
+      <c r="H3613">
+        <v>75.900000000000006</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Rerun results after corrected June 2026 data
</commit_message>
<xml_diff>
--- a/date_simp_concat.xlsx
+++ b/date_simp_concat.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Desktop\Doctorat\simpozion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{432710BF-29F3-45A3-BD91-BBB3BCCBB788}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC851B6D-316F-4EEC-865C-AB19C074C2A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -92152,7 +92152,7 @@
         <v>46056</v>
       </c>
       <c r="B3529">
-        <v>226.48</v>
+        <v>225.62</v>
       </c>
       <c r="C3529">
         <v>617.92999999999995</v>
@@ -92178,7 +92178,7 @@
         <v>46057</v>
       </c>
       <c r="B3530">
-        <v>225.43</v>
+        <v>225.76</v>
       </c>
       <c r="C3530">
         <v>618.12</v>
@@ -92204,7 +92204,7 @@
         <v>46058</v>
       </c>
       <c r="B3531">
-        <v>225.65</v>
+        <v>223.65</v>
       </c>
       <c r="C3531">
         <v>611.65</v>
@@ -92230,7 +92230,7 @@
         <v>46059</v>
       </c>
       <c r="B3532">
-        <v>223.53</v>
+        <v>225.46</v>
       </c>
       <c r="C3532">
         <v>617.12</v>
@@ -92256,7 +92256,7 @@
         <v>46062</v>
       </c>
       <c r="B3533">
-        <v>225.77</v>
+        <v>226.84</v>
       </c>
       <c r="C3533">
         <v>621.41</v>
@@ -92282,7 +92282,7 @@
         <v>46063</v>
       </c>
       <c r="B3534">
-        <v>226.99</v>
+        <v>226.98</v>
       </c>
       <c r="C3534">
         <v>620.97</v>
@@ -92308,7 +92308,7 @@
         <v>46064</v>
       </c>
       <c r="B3535">
-        <v>226.81</v>
+        <v>227</v>
       </c>
       <c r="C3535">
         <v>621.58000000000004</v>
@@ -92334,7 +92334,7 @@
         <v>46065</v>
       </c>
       <c r="B3536">
-        <v>227.78</v>
+        <v>225.97</v>
       </c>
       <c r="C3536">
         <v>618.52</v>
@@ -92360,7 +92360,7 @@
         <v>46066</v>
       </c>
       <c r="B3537">
-        <v>225.96</v>
+        <v>225.29</v>
       </c>
       <c r="C3537">
         <v>617.70000000000005</v>
@@ -92386,7 +92386,7 @@
         <v>46069</v>
       </c>
       <c r="B3538">
-        <v>225.83</v>
+        <v>225.45</v>
       </c>
       <c r="C3538">
         <v>618.52</v>
@@ -92412,7 +92412,7 @@
         <v>46070</v>
       </c>
       <c r="B3539">
-        <v>225.19</v>
+        <v>226.68</v>
       </c>
       <c r="C3539">
         <v>621.29</v>
@@ -92438,7 +92438,7 @@
         <v>46071</v>
       </c>
       <c r="B3540">
-        <v>227.08</v>
+        <v>228.98</v>
       </c>
       <c r="C3540">
         <v>628.69000000000005</v>
@@ -92464,7 +92464,7 @@
         <v>46072</v>
       </c>
       <c r="B3541">
-        <v>228.98</v>
+        <v>227.57</v>
       </c>
       <c r="C3541">
         <v>625.33000000000004</v>
@@ -92490,7 +92490,7 @@
         <v>46073</v>
       </c>
       <c r="B3542">
-        <v>228.05</v>
+        <v>229.69</v>
       </c>
       <c r="C3542">
         <v>630.55999999999995</v>
@@ -92516,7 +92516,7 @@
         <v>46076</v>
       </c>
       <c r="B3543">
-        <v>229.36</v>
+        <v>228.63</v>
       </c>
       <c r="C3543">
         <v>627.70000000000005</v>
@@ -92542,7 +92542,7 @@
         <v>46077</v>
       </c>
       <c r="B3544">
-        <v>228.56</v>
+        <v>229.19</v>
       </c>
       <c r="C3544">
         <v>629.14</v>
@@ -92568,7 +92568,7 @@
         <v>46078</v>
       </c>
       <c r="B3545">
-        <v>229.67</v>
+        <v>230.9</v>
       </c>
       <c r="C3545">
         <v>633.47</v>
@@ -92594,7 +92594,7 @@
         <v>46079</v>
       </c>
       <c r="B3546">
-        <v>230.89</v>
+        <v>230.69</v>
       </c>
       <c r="C3546">
         <v>633.17999999999995</v>
@@ -92620,7 +92620,7 @@
         <v>46080</v>
       </c>
       <c r="B3547">
-        <v>230.64</v>
+        <v>231.14</v>
       </c>
       <c r="C3547">
         <v>633.85</v>
@@ -92646,7 +92646,7 @@
         <v>46083</v>
       </c>
       <c r="B3548">
-        <v>228.71</v>
+        <v>226.52</v>
       </c>
       <c r="C3548">
         <v>623.63</v>
@@ -92672,7 +92672,7 @@
         <v>46084</v>
       </c>
       <c r="B3549">
-        <v>225.13</v>
+        <v>219.22</v>
       </c>
       <c r="C3549">
         <v>604.44000000000005</v>
@@ -92698,7 +92698,7 @@
         <v>46085</v>
       </c>
       <c r="B3550">
-        <v>219.64</v>
+        <v>222.41</v>
       </c>
       <c r="C3550">
         <v>612.71</v>
@@ -92724,7 +92724,7 @@
         <v>46086</v>
       </c>
       <c r="B3551">
-        <v>222.39</v>
+        <v>219.62</v>
       </c>
       <c r="C3551">
         <v>604.83000000000004</v>
@@ -92750,7 +92750,7 @@
         <v>46087</v>
       </c>
       <c r="B3552">
-        <v>220.44</v>
+        <v>216.87</v>
       </c>
       <c r="C3552">
         <v>598.69000000000005</v>
@@ -92776,7 +92776,7 @@
         <v>46090</v>
       </c>
       <c r="B3553">
-        <v>214.75</v>
+        <v>215.05</v>
       </c>
       <c r="C3553">
         <v>594.91999999999996</v>
@@ -92802,7 +92802,7 @@
         <v>46091</v>
       </c>
       <c r="B3554">
-        <v>216.32</v>
+        <v>219.31</v>
       </c>
       <c r="C3554">
         <v>606.12</v>
@@ -92828,7 +92828,7 @@
         <v>46092</v>
       </c>
       <c r="B3555">
-        <v>218.58</v>
+        <v>217.83</v>
       </c>
       <c r="C3555">
         <v>602.54</v>
@@ -92854,7 +92854,7 @@
         <v>46093</v>
       </c>
       <c r="B3556">
-        <v>217.18</v>
+        <v>216</v>
       </c>
       <c r="C3556">
         <v>598.86</v>
@@ -92880,7 +92880,7 @@
         <v>46094</v>
       </c>
       <c r="B3557">
-        <v>215.2</v>
+        <v>214.84</v>
       </c>
       <c r="C3557">
         <v>595.85</v>
@@ -92906,7 +92906,7 @@
         <v>46097</v>
       </c>
       <c r="B3558">
-        <v>214.86</v>
+        <v>215.63</v>
       </c>
       <c r="C3558">
         <v>598.47</v>
@@ -92932,7 +92932,7 @@
         <v>46098</v>
       </c>
       <c r="B3559">
-        <v>215.54</v>
+        <v>216.9</v>
       </c>
       <c r="C3559">
         <v>602.45000000000005</v>
@@ -92958,7 +92958,7 @@
         <v>46099</v>
       </c>
       <c r="B3560">
-        <v>217.42</v>
+        <v>215.02</v>
       </c>
       <c r="C3560">
         <v>597.92999999999995</v>
@@ -92984,7 +92984,7 @@
         <v>46100</v>
       </c>
       <c r="B3561">
-        <v>213.56</v>
+        <v>209.29</v>
       </c>
       <c r="C3561">
         <v>583.64</v>
@@ -93010,7 +93010,7 @@
         <v>46101</v>
       </c>
       <c r="B3562">
-        <v>210.35</v>
+        <v>205.74</v>
       </c>
       <c r="C3562">
         <v>573.28</v>
@@ -93036,7 +93036,7 @@
         <v>46104</v>
       </c>
       <c r="B3563">
-        <v>204.19</v>
+        <v>207.48</v>
       </c>
       <c r="C3563">
         <v>576.78</v>
@@ -93062,7 +93062,7 @@
         <v>46105</v>
       </c>
       <c r="B3564">
-        <v>207.82</v>
+        <v>208.29</v>
       </c>
       <c r="C3564">
         <v>579.28</v>
@@ -93088,7 +93088,7 @@
         <v>46106</v>
       </c>
       <c r="B3565">
-        <v>209.21</v>
+        <v>211.29</v>
       </c>
       <c r="C3565">
         <v>587.49</v>
@@ -93114,7 +93114,7 @@
         <v>46107</v>
       </c>
       <c r="B3566">
-        <v>210.41</v>
+        <v>208.62</v>
       </c>
       <c r="C3566">
         <v>580.84</v>
@@ -93140,7 +93140,7 @@
         <v>46108</v>
       </c>
       <c r="B3567">
-        <v>208.7</v>
+        <v>206.7</v>
       </c>
       <c r="C3567">
         <v>575.29999999999995</v>
@@ -93166,7 +93166,7 @@
         <v>46111</v>
       </c>
       <c r="B3568">
-        <v>206.35</v>
+        <v>208.48</v>
       </c>
       <c r="C3568">
         <v>580.73</v>
@@ -93192,7 +93192,7 @@
         <v>46112</v>
       </c>
       <c r="B3569">
-        <v>208.62</v>
+        <v>209.17</v>
       </c>
       <c r="C3569">
         <v>583.14</v>
@@ -93218,7 +93218,7 @@
         <v>46113</v>
       </c>
       <c r="B3570">
-        <v>211.35</v>
+        <v>215.02</v>
       </c>
       <c r="C3570">
         <v>597.69000000000005</v>
@@ -93244,7 +93244,7 @@
         <v>46114</v>
       </c>
       <c r="B3571">
-        <v>213.27</v>
+        <v>214.3</v>
       </c>
       <c r="C3571">
         <v>596.63</v>
@@ -93270,7 +93270,7 @@
         <v>46119</v>
       </c>
       <c r="B3572">
-        <v>214.81</v>
+        <v>212.03</v>
       </c>
       <c r="C3572">
         <v>590.59</v>
@@ -93296,7 +93296,7 @@
         <v>46120</v>
       </c>
       <c r="B3573">
-        <v>214.16</v>
+        <v>221.19</v>
       </c>
       <c r="C3573">
         <v>613.5</v>
@@ -93322,7 +93322,7 @@
         <v>46121</v>
       </c>
       <c r="B3574">
-        <v>220.82</v>
+        <v>220.65</v>
       </c>
       <c r="C3574">
         <v>612.59</v>
@@ -93348,7 +93348,7 @@
         <v>46122</v>
       </c>
       <c r="B3575">
-        <v>220.82</v>
+        <v>221.94</v>
       </c>
       <c r="C3575">
         <v>614.84</v>
@@ -93374,7 +93374,7 @@
         <v>46125</v>
       </c>
       <c r="B3576">
-        <v>220.96</v>
+        <v>221.25</v>
       </c>
       <c r="C3576">
         <v>613.88</v>
@@ -93400,7 +93400,7 @@
         <v>46126</v>
       </c>
       <c r="B3577">
-        <v>221.72</v>
+        <v>223.98</v>
       </c>
       <c r="C3577">
         <v>619.95000000000005</v>
@@ -93426,7 +93426,7 @@
         <v>46127</v>
       </c>
       <c r="B3578">
-        <v>224.1</v>
+        <v>223.08</v>
       </c>
       <c r="C3578">
         <v>617.27</v>
@@ -93452,7 +93452,7 @@
         <v>46128</v>
       </c>
       <c r="B3579">
-        <v>223.3</v>
+        <v>223.08</v>
       </c>
       <c r="C3579">
         <v>616.95000000000005</v>
@@ -93478,7 +93478,7 @@
         <v>46129</v>
       </c>
       <c r="B3580">
-        <v>222.64</v>
+        <v>227.38</v>
       </c>
       <c r="C3580">
         <v>626.58000000000004</v>
@@ -93504,7 +93504,7 @@
         <v>46132</v>
       </c>
       <c r="B3581">
-        <v>225.56</v>
+        <v>225.2</v>
       </c>
       <c r="C3581">
         <v>621.46</v>
@@ -93530,7 +93530,7 @@
         <v>46133</v>
       </c>
       <c r="B3582">
-        <v>225.43</v>
+        <v>223.55</v>
       </c>
       <c r="C3582">
         <v>616.03</v>
@@ -93556,7 +93556,7 @@
         <v>46134</v>
       </c>
       <c r="B3583">
-        <v>223.89</v>
+        <v>222.7</v>
       </c>
       <c r="C3583">
         <v>613.88</v>
@@ -93582,7 +93582,7 @@
         <v>46135</v>
       </c>
       <c r="B3584">
-        <v>222.02</v>
+        <v>222.62</v>
       </c>
       <c r="C3584">
         <v>614.20000000000005</v>
@@ -93608,7 +93608,7 @@
         <v>46136</v>
       </c>
       <c r="B3585">
-        <v>221.88</v>
+        <v>221.6</v>
       </c>
       <c r="C3585">
         <v>610.65</v>
@@ -93634,7 +93634,7 @@
         <v>46139</v>
       </c>
       <c r="B3586">
-        <v>221.53</v>
+        <v>220.88</v>
       </c>
       <c r="C3586">
         <v>608.84</v>
@@ -93660,7 +93660,7 @@
         <v>46140</v>
       </c>
       <c r="B3587">
-        <v>220.57</v>
+        <v>219.9</v>
       </c>
       <c r="C3587">
         <v>606.58000000000004</v>
@@ -93686,7 +93686,7 @@
         <v>46141</v>
       </c>
       <c r="B3588">
-        <v>220.04</v>
+        <v>218.49</v>
       </c>
       <c r="C3588">
         <v>602.96</v>
@@ -93712,7 +93712,7 @@
         <v>46142</v>
       </c>
       <c r="B3589">
-        <v>217.31</v>
+        <v>221.25</v>
       </c>
       <c r="C3589">
         <v>611.28</v>
@@ -93738,7 +93738,7 @@
         <v>46146</v>
       </c>
       <c r="B3590">
-        <v>221.46</v>
+        <v>218.82</v>
       </c>
       <c r="C3590">
         <v>605.51</v>
@@ -93764,7 +93764,7 @@
         <v>46147</v>
       </c>
       <c r="B3591">
-        <v>218.63</v>
+        <v>220.36</v>
       </c>
       <c r="C3591">
         <v>609.72</v>
@@ -93790,7 +93790,7 @@
         <v>46148</v>
       </c>
       <c r="B3592">
-        <v>221.23</v>
+        <v>225.7</v>
       </c>
       <c r="C3592">
         <v>623.25</v>
@@ -93816,7 +93816,7 @@
         <v>46149</v>
       </c>
       <c r="B3593">
-        <v>225.9</v>
+        <v>223.56</v>
       </c>
       <c r="C3593">
         <v>616.41999999999996</v>
@@ -93842,7 +93842,7 @@
         <v>46150</v>
       </c>
       <c r="B3594">
-        <v>222.76</v>
+        <v>222.24</v>
       </c>
       <c r="C3594">
         <v>612.14</v>
@@ -93868,7 +93868,7 @@
         <v>46153</v>
       </c>
       <c r="B3595">
-        <v>222.16</v>
+        <v>222.35</v>
       </c>
       <c r="C3595">
         <v>612.79</v>
@@ -93894,7 +93894,7 @@
         <v>46154</v>
       </c>
       <c r="B3596">
-        <v>220.79</v>
+        <v>219.74</v>
       </c>
       <c r="C3596">
         <v>606.63</v>
@@ -93920,7 +93920,7 @@
         <v>46155</v>
       </c>
       <c r="B3597">
-        <v>220.49</v>
+        <v>221.68</v>
       </c>
       <c r="C3597">
         <v>611.41999999999996</v>
@@ -93946,7 +93946,7 @@
         <v>46156</v>
       </c>
       <c r="B3598">
-        <v>222.07</v>
+        <v>223.5</v>
       </c>
       <c r="C3598">
         <v>616.04999999999995</v>
@@ -93972,7 +93972,7 @@
         <v>46157</v>
       </c>
       <c r="B3599">
-        <v>222.68</v>
+        <v>220.2</v>
       </c>
       <c r="C3599">
         <v>606.91999999999996</v>
@@ -93998,7 +93998,7 @@
         <v>46160</v>
       </c>
       <c r="B3600">
-        <v>219.22</v>
+        <v>220.95</v>
       </c>
       <c r="C3600">
         <v>610.16999999999996</v>
@@ -94024,7 +94024,7 @@
         <v>46161</v>
       </c>
       <c r="B3601">
-        <v>221.17</v>
+        <v>221.35</v>
       </c>
       <c r="C3601">
         <v>611.34</v>
@@ -94050,7 +94050,7 @@
         <v>46162</v>
       </c>
       <c r="B3602">
-        <v>221.15</v>
+        <v>224.7</v>
       </c>
       <c r="C3602">
         <v>620.29</v>
@@ -94076,7 +94076,7 @@
         <v>46163</v>
       </c>
       <c r="B3603">
-        <v>224.45</v>
+        <v>224.9</v>
       </c>
       <c r="C3603">
         <v>620.55999999999995</v>
@@ -94102,7 +94102,7 @@
         <v>46164</v>
       </c>
       <c r="B3604">
-        <v>225.7</v>
+        <v>226.8</v>
       </c>
       <c r="C3604">
         <v>625.12</v>
@@ -94128,7 +94128,7 @@
         <v>46168</v>
       </c>
       <c r="B3605">
-        <v>229.22</v>
+        <v>227.92</v>
       </c>
       <c r="C3605">
         <v>628.01</v>
@@ -94154,7 +94154,7 @@
         <v>46169</v>
       </c>
       <c r="B3606">
-        <v>227.92</v>
+        <v>228.26</v>
       </c>
       <c r="C3606">
         <v>628.17999999999995</v>
@@ -94180,7 +94180,7 @@
         <v>46170</v>
       </c>
       <c r="B3607">
-        <v>227.63</v>
+        <v>226.69</v>
       </c>
       <c r="C3607">
         <v>625.11</v>
@@ -94206,7 +94206,7 @@
         <v>46171</v>
       </c>
       <c r="B3608">
-        <v>227.03</v>
+        <v>227</v>
       </c>
       <c r="C3608">
         <v>626</v>
@@ -94232,7 +94232,7 @@
         <v>46174</v>
       </c>
       <c r="B3609">
-        <v>226.91</v>
+        <v>225.25</v>
       </c>
       <c r="C3609">
         <v>621.24</v>
@@ -94258,7 +94258,7 @@
         <v>46175</v>
       </c>
       <c r="B3610">
-        <v>225.95</v>
+        <v>227.05</v>
       </c>
       <c r="C3610">
         <v>625.34</v>
@@ -94284,7 +94284,7 @@
         <v>46176</v>
       </c>
       <c r="B3611">
-        <v>226.89</v>
+        <v>225.33</v>
       </c>
       <c r="C3611">
         <v>621.19000000000005</v>
@@ -94310,7 +94310,7 @@
         <v>46177</v>
       </c>
       <c r="B3612">
-        <v>225.27</v>
+        <v>226.67</v>
       </c>
       <c r="C3612">
         <v>624.45000000000005</v>
@@ -94336,7 +94336,7 @@
         <v>46178</v>
       </c>
       <c r="B3613">
-        <v>226.77</v>
+        <v>225.84</v>
       </c>
       <c r="C3613">
         <v>622.66</v>

</xml_diff>